<commit_message>
Add kids to admin export
</commit_message>
<xml_diff>
--- a/backend/platform/src/main/resources/jxls/admin_employees_template.xlsx
+++ b/backend/platform/src/main/resources/jxls/admin_employees_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873A185E-000B-4844-9EB0-EB38AC64A977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24263E7-AB49-442A-AA60-D4DC097CD539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Сотрудники" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="2" r:id="rId2"/>
+    <sheet name="Сотрудники" sheetId="3" r:id="rId1"/>
+    <sheet name="Дети" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,6 +27,64 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Автор</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4E4EC45D-AC2B-4104-B883-BA69106E8CAA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Автор:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+jx:area(lastCell="Z4")</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{E99472F8-9A50-4721-A7AF-B453FD4ADFD8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Автор:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+jx:each(items="employees" var="e" lastCell="Z4" orderBy="displayName")</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Автор</author>
@@ -52,7 +110,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:area(lastCell="AA4")</t>
+jx:area(lastCell="E4")</t>
         </r>
       </text>
     </comment>
@@ -76,7 +134,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:each(items="employees" var="e" lastCell="AA4" orderBy="displayName")</t>
+jx:each(items="kids" var="kid" lastCell="E4" orderBy="parent.displayName")</t>
         </r>
       </text>
     </comment>
@@ -85,7 +143,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="66">
   <si>
     <t>ФИО</t>
   </si>
@@ -111,12 +169,6 @@
     <t>${e.phone}</t>
   </si>
   <si>
-    <t>Skype</t>
-  </si>
-  <si>
-    <t>${e.skype}</t>
-  </si>
-  <si>
     <t>Дата трудоустройства</t>
   </si>
   <si>
@@ -256,6 +308,39 @@
   </si>
   <si>
     <t>${e.organization}</t>
+  </si>
+  <si>
+    <t>Выгрузка детей сотрудников компании из системы HR Easy</t>
+  </si>
+  <si>
+    <t>ФИО сотрудника</t>
+  </si>
+  <si>
+    <t>Email сотрудника</t>
+  </si>
+  <si>
+    <t>Имя ребёнка</t>
+  </si>
+  <si>
+    <t>Дата рождения</t>
+  </si>
+  <si>
+    <t>Возраст</t>
+  </si>
+  <si>
+    <t>${kid.displayName}</t>
+  </si>
+  <si>
+    <t>${kid.birthday}</t>
+  </si>
+  <si>
+    <t>${kid.age}</t>
+  </si>
+  <si>
+    <t>${kid.parent.displayName}</t>
+  </si>
+  <si>
+    <t>${kid.parent.email}</t>
   </si>
 </sst>
 </file>
@@ -382,30 +467,9 @@
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+  <dxfs count="17">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -441,6 +505,64 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE84C05"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -460,6 +582,54 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2095500</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>171100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15F3D519-6E4D-47F0-A414-5074DFDFEA8D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect l="2979" t="8904" r="4679" b="13698"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="504825" y="0"/>
+          <a:ext cx="1590675" cy="828325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -508,48 +678,64 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A3:AA4" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A3:AA4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AA4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E44C5C4F-FB14-43F8-AA75-45270F5135AF}" name="Таблица13" displayName="Таблица13" ref="A3:Z4" totalsRowShown="0" headerRowDxfId="16">
+  <autoFilter ref="A3:Z4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:Z4">
     <sortCondition ref="A3:A4"/>
   </sortState>
-  <tableColumns count="27">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ФИО"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Текущий проект" dataDxfId="9"/>
-    <tableColumn id="26" xr3:uid="{2CF1E783-42FA-435B-A9B0-71CCC889D77B}" name="Роль на проекте" dataDxfId="8"/>
-    <tableColumn id="24" xr3:uid="{D293F5E8-02A4-47F1-A8B5-1446B2110421}" name="Бизнес аккаунт" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Телефон" dataDxfId="6"/>
-    <tableColumn id="25" xr3:uid="{3DBEBAD8-1961-454B-AB1D-54B4D3044F8A}" name="Telegram" dataDxfId="5"/>
-    <tableColumn id="27" xr3:uid="{10B83D6D-F71C-42A9-9640-B2DC46318818}" name="Подразделение" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{4E765C0B-EC7F-4DD0-9E45-AA769E6594A7}" name="Организация" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Дата трудоустройства" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="День рождения" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Позиция"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Уровень экспертизы"/>
-    <tableColumn id="10" xr3:uid="{DA50F1B3-475E-4D76-9C0A-64F0B8D65742}" name="Рабочее место"/>
-    <tableColumn id="11" xr3:uid="{8C711430-DA03-4D17-9A2B-66F6DEB83EB0}" name="Документ УЛ"/>
-    <tableColumn id="12" xr3:uid="{660D3940-252F-4179-9D86-3BBA1CC7D76F}" name="Адрес по регистрации"/>
-    <tableColumn id="13" xr3:uid="{171FA4C5-9876-48E9-8A8D-8F46602A3C98}" name="Пол"/>
-    <tableColumn id="14" xr3:uid="{C544F49F-228C-43BC-A19B-2358B1C43905}" name="ФИО супруга/супруги"/>
-    <tableColumn id="15" xr3:uid="{AAC3EF14-AB7F-4E28-B27A-D4BB5C3FEED4}" name="Рабочий день"/>
-    <tableColumn id="16" xr3:uid="{B39AB8F8-F9A7-44C7-BB9F-896266D2AF17}" name="Место работы"/>
-    <tableColumn id="18" xr3:uid="{C27F935E-18D9-4D42-8EF2-7F711FFE8654}" name="Город проживания"/>
-    <tableColumn id="19" xr3:uid="{2C11CA5F-E5AC-4676-8068-44894FCD3D15}" name="Дети"/>
-    <tableColumn id="20" xr3:uid="{A17EE04E-E8C8-477E-AF16-C735D4063995}" name="Семейный статус"/>
-    <tableColumn id="21" xr3:uid="{79B291B5-5726-498B-B004-5B1A54643FBC}" name="Загранпаспорт"/>
-    <tableColumn id="22" xr3:uid="{3EC984DC-1A99-4FDD-BEFC-E6ADF5BBF9E7}" name="Уровень английского"/>
-    <tableColumn id="28" xr3:uid="{AC770C52-4960-4CFD-B50D-CFB1613486F1}" name="Skype"/>
-    <tableColumn id="23" xr3:uid="{13E7F2B1-140C-43F9-AD05-47E67B04BB41}" name="Дата увольнения" dataDxfId="2"/>
+  <tableColumns count="26">
+    <tableColumn id="1" xr3:uid="{8EE2DE2E-7CC4-459D-B0CA-6E2E931061CB}" name="ФИО"/>
+    <tableColumn id="2" xr3:uid="{686E9D29-1F6A-4301-953F-F8F65FC9F4C4}" name="Email" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{E11EF56B-FA6A-4875-B62E-0C7B2757DD5F}" name="Текущий проект" dataDxfId="14"/>
+    <tableColumn id="26" xr3:uid="{DEA09456-5F8F-41E6-8A9B-7ADBE17A6F5B}" name="Роль на проекте" dataDxfId="13"/>
+    <tableColumn id="24" xr3:uid="{3FA3F769-10F5-48FD-9962-CF3B7E203181}" name="Бизнес аккаунт" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{DB6376FB-06A6-4916-A4C9-E64078E7284D}" name="Телефон" dataDxfId="11"/>
+    <tableColumn id="25" xr3:uid="{192DBCFF-41C4-45A9-905E-532722BA700F}" name="Telegram" dataDxfId="10"/>
+    <tableColumn id="27" xr3:uid="{4CBDC5CD-8D5A-49FA-B362-A2E3E38D577A}" name="Подразделение" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{9D8E3AF1-45DC-46AE-B9D8-571CF57CAA0F}" name="Организация" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{5F6082CD-D37C-496D-BFF0-50E633B09001}" name="Дата трудоустройства" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{DF0A2FF2-3D40-492B-A0EF-FB7C98C5F19C}" name="День рождения" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{9F36C173-64FF-441B-8861-40062D26EC5F}" name="Позиция"/>
+    <tableColumn id="9" xr3:uid="{D312A1E1-7C2E-4D8A-944A-4F3689255C0C}" name="Уровень экспертизы"/>
+    <tableColumn id="10" xr3:uid="{7AE2A8AB-0688-4A8B-8012-028FAC792776}" name="Рабочее место"/>
+    <tableColumn id="11" xr3:uid="{E00E5D5B-B0D7-4D3E-8330-D83170ECDFFD}" name="Документ УЛ"/>
+    <tableColumn id="12" xr3:uid="{7856E0FF-220B-4C61-A0A9-7F69D6EEC19E}" name="Адрес по регистрации"/>
+    <tableColumn id="13" xr3:uid="{44810D1B-1CF3-4DCF-83FF-EA7B1EED8C28}" name="Пол"/>
+    <tableColumn id="14" xr3:uid="{AD618D33-9F1F-4128-82F7-EFFB19B34980}" name="ФИО супруга/супруги"/>
+    <tableColumn id="15" xr3:uid="{8E247D4A-8763-4FAF-A7A3-EC126825E3BF}" name="Рабочий день"/>
+    <tableColumn id="16" xr3:uid="{B1BA21C0-74F6-4B20-9CB0-AD84D7F04623}" name="Место работы"/>
+    <tableColumn id="18" xr3:uid="{6AFC2477-2AC6-4181-97C1-55DE239AB899}" name="Город проживания"/>
+    <tableColumn id="19" xr3:uid="{5B31A27F-B1A8-49A9-85BF-1C34811AF3DC}" name="Дети"/>
+    <tableColumn id="20" xr3:uid="{512F8F09-CC0D-4E0A-93C2-9B4E67614C53}" name="Семейный статус"/>
+    <tableColumn id="21" xr3:uid="{AD98EEC2-5FB0-4A32-969B-092FF90D08BC}" name="Загранпаспорт"/>
+    <tableColumn id="22" xr3:uid="{213A8395-60CF-4627-8BFA-8B7932AB04B3}" name="Уровень английского"/>
+    <tableColumn id="23" xr3:uid="{2B2BC760-206D-4B47-91E1-3A23B46C94A0}" name="Дата увольнения" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A3:E4" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A3:E4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:E4">
+    <sortCondition ref="A3:A4"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ФИО сотрудника"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email сотрудника" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Имя ребёнка" dataDxfId="2"/>
+    <tableColumn id="26" xr3:uid="{2CF1E783-42FA-435B-A9B0-71CCC889D77B}" name="Дата рождения" dataDxfId="0"/>
+    <tableColumn id="24" xr3:uid="{D293F5E8-02A4-47F1-A8B5-1446B2110421}" name="Возраст" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Стандартная">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -587,9 +773,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -622,9 +808,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -657,9 +860,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Стандартная">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -832,8 +1052,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F76F545-ACAE-4135-9050-AC0BC6DE98B0}">
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.5703125" customWidth="1"/>
@@ -860,10 +1080,10 @@
     <col min="24" max="24" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5"/>
       <c r="B1" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -888,7 +1108,7 @@
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="9" t="s">
         <v>1</v>
@@ -918,7 +1138,7 @@
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
     </row>
-    <row r="3" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -929,159 +1149,153 @@
         <v>3</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="V3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="U3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="X3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="Y3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="X3" s="4" t="s">
+      <c r="Z3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Y3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>31</v>
-      </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" t="s">
+        <v>43</v>
+      </c>
+      <c r="O4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S4" t="s">
         <v>38</v>
       </c>
-      <c r="I4" t="s">
-        <v>56</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" t="s">
-        <v>45</v>
-      </c>
-      <c r="O4" t="s">
-        <v>44</v>
-      </c>
-      <c r="P4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>42</v>
-      </c>
-      <c r="R4" t="s">
-        <v>41</v>
-      </c>
-      <c r="S4" t="s">
-        <v>40</v>
-      </c>
       <c r="T4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="U4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="V4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="W4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="X4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Y4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA4" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="Z4" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1096,10 +1310,77 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CA4589C-B720-4D4E-AE1C-33C6E71A124A}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="41.5703125" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="39.42578125" customWidth="1"/>
+    <col min="4" max="5" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
External API improvments (#106)
* Remove internal ids from external api
* Add ability to make project workstream required
* Add kids to admin export
</commit_message>
<xml_diff>
--- a/backend/platform/src/main/resources/jxls/admin_employees_template.xlsx
+++ b/backend/platform/src/main/resources/jxls/admin_employees_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873A185E-000B-4844-9EB0-EB38AC64A977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24263E7-AB49-442A-AA60-D4DC097CD539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Сотрудники" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="2" r:id="rId2"/>
+    <sheet name="Сотрудники" sheetId="3" r:id="rId1"/>
+    <sheet name="Дети" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,6 +27,64 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Автор</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4E4EC45D-AC2B-4104-B883-BA69106E8CAA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Автор:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+jx:area(lastCell="Z4")</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{E99472F8-9A50-4721-A7AF-B453FD4ADFD8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Автор:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+jx:each(items="employees" var="e" lastCell="Z4" orderBy="displayName")</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Автор</author>
@@ -52,7 +110,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:area(lastCell="AA4")</t>
+jx:area(lastCell="E4")</t>
         </r>
       </text>
     </comment>
@@ -76,7 +134,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-jx:each(items="employees" var="e" lastCell="AA4" orderBy="displayName")</t>
+jx:each(items="kids" var="kid" lastCell="E4" orderBy="parent.displayName")</t>
         </r>
       </text>
     </comment>
@@ -85,7 +143,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="66">
   <si>
     <t>ФИО</t>
   </si>
@@ -111,12 +169,6 @@
     <t>${e.phone}</t>
   </si>
   <si>
-    <t>Skype</t>
-  </si>
-  <si>
-    <t>${e.skype}</t>
-  </si>
-  <si>
     <t>Дата трудоустройства</t>
   </si>
   <si>
@@ -256,6 +308,39 @@
   </si>
   <si>
     <t>${e.organization}</t>
+  </si>
+  <si>
+    <t>Выгрузка детей сотрудников компании из системы HR Easy</t>
+  </si>
+  <si>
+    <t>ФИО сотрудника</t>
+  </si>
+  <si>
+    <t>Email сотрудника</t>
+  </si>
+  <si>
+    <t>Имя ребёнка</t>
+  </si>
+  <si>
+    <t>Дата рождения</t>
+  </si>
+  <si>
+    <t>Возраст</t>
+  </si>
+  <si>
+    <t>${kid.displayName}</t>
+  </si>
+  <si>
+    <t>${kid.birthday}</t>
+  </si>
+  <si>
+    <t>${kid.age}</t>
+  </si>
+  <si>
+    <t>${kid.parent.displayName}</t>
+  </si>
+  <si>
+    <t>${kid.parent.email}</t>
   </si>
 </sst>
 </file>
@@ -382,30 +467,9 @@
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+  <dxfs count="17">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -441,6 +505,64 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE84C05"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -460,6 +582,54 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2095500</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>171100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15F3D519-6E4D-47F0-A414-5074DFDFEA8D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect l="2979" t="8904" r="4679" b="13698"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="504825" y="0"/>
+          <a:ext cx="1590675" cy="828325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -508,48 +678,64 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A3:AA4" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A3:AA4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AA4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E44C5C4F-FB14-43F8-AA75-45270F5135AF}" name="Таблица13" displayName="Таблица13" ref="A3:Z4" totalsRowShown="0" headerRowDxfId="16">
+  <autoFilter ref="A3:Z4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:Z4">
     <sortCondition ref="A3:A4"/>
   </sortState>
-  <tableColumns count="27">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ФИО"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Текущий проект" dataDxfId="9"/>
-    <tableColumn id="26" xr3:uid="{2CF1E783-42FA-435B-A9B0-71CCC889D77B}" name="Роль на проекте" dataDxfId="8"/>
-    <tableColumn id="24" xr3:uid="{D293F5E8-02A4-47F1-A8B5-1446B2110421}" name="Бизнес аккаунт" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Телефон" dataDxfId="6"/>
-    <tableColumn id="25" xr3:uid="{3DBEBAD8-1961-454B-AB1D-54B4D3044F8A}" name="Telegram" dataDxfId="5"/>
-    <tableColumn id="27" xr3:uid="{10B83D6D-F71C-42A9-9640-B2DC46318818}" name="Подразделение" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{4E765C0B-EC7F-4DD0-9E45-AA769E6594A7}" name="Организация" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Дата трудоустройства" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="День рождения" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Позиция"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Уровень экспертизы"/>
-    <tableColumn id="10" xr3:uid="{DA50F1B3-475E-4D76-9C0A-64F0B8D65742}" name="Рабочее место"/>
-    <tableColumn id="11" xr3:uid="{8C711430-DA03-4D17-9A2B-66F6DEB83EB0}" name="Документ УЛ"/>
-    <tableColumn id="12" xr3:uid="{660D3940-252F-4179-9D86-3BBA1CC7D76F}" name="Адрес по регистрации"/>
-    <tableColumn id="13" xr3:uid="{171FA4C5-9876-48E9-8A8D-8F46602A3C98}" name="Пол"/>
-    <tableColumn id="14" xr3:uid="{C544F49F-228C-43BC-A19B-2358B1C43905}" name="ФИО супруга/супруги"/>
-    <tableColumn id="15" xr3:uid="{AAC3EF14-AB7F-4E28-B27A-D4BB5C3FEED4}" name="Рабочий день"/>
-    <tableColumn id="16" xr3:uid="{B39AB8F8-F9A7-44C7-BB9F-896266D2AF17}" name="Место работы"/>
-    <tableColumn id="18" xr3:uid="{C27F935E-18D9-4D42-8EF2-7F711FFE8654}" name="Город проживания"/>
-    <tableColumn id="19" xr3:uid="{2C11CA5F-E5AC-4676-8068-44894FCD3D15}" name="Дети"/>
-    <tableColumn id="20" xr3:uid="{A17EE04E-E8C8-477E-AF16-C735D4063995}" name="Семейный статус"/>
-    <tableColumn id="21" xr3:uid="{79B291B5-5726-498B-B004-5B1A54643FBC}" name="Загранпаспорт"/>
-    <tableColumn id="22" xr3:uid="{3EC984DC-1A99-4FDD-BEFC-E6ADF5BBF9E7}" name="Уровень английского"/>
-    <tableColumn id="28" xr3:uid="{AC770C52-4960-4CFD-B50D-CFB1613486F1}" name="Skype"/>
-    <tableColumn id="23" xr3:uid="{13E7F2B1-140C-43F9-AD05-47E67B04BB41}" name="Дата увольнения" dataDxfId="2"/>
+  <tableColumns count="26">
+    <tableColumn id="1" xr3:uid="{8EE2DE2E-7CC4-459D-B0CA-6E2E931061CB}" name="ФИО"/>
+    <tableColumn id="2" xr3:uid="{686E9D29-1F6A-4301-953F-F8F65FC9F4C4}" name="Email" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{E11EF56B-FA6A-4875-B62E-0C7B2757DD5F}" name="Текущий проект" dataDxfId="14"/>
+    <tableColumn id="26" xr3:uid="{DEA09456-5F8F-41E6-8A9B-7ADBE17A6F5B}" name="Роль на проекте" dataDxfId="13"/>
+    <tableColumn id="24" xr3:uid="{3FA3F769-10F5-48FD-9962-CF3B7E203181}" name="Бизнес аккаунт" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{DB6376FB-06A6-4916-A4C9-E64078E7284D}" name="Телефон" dataDxfId="11"/>
+    <tableColumn id="25" xr3:uid="{192DBCFF-41C4-45A9-905E-532722BA700F}" name="Telegram" dataDxfId="10"/>
+    <tableColumn id="27" xr3:uid="{4CBDC5CD-8D5A-49FA-B362-A2E3E38D577A}" name="Подразделение" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{9D8E3AF1-45DC-46AE-B9D8-571CF57CAA0F}" name="Организация" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{5F6082CD-D37C-496D-BFF0-50E633B09001}" name="Дата трудоустройства" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{DF0A2FF2-3D40-492B-A0EF-FB7C98C5F19C}" name="День рождения" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{9F36C173-64FF-441B-8861-40062D26EC5F}" name="Позиция"/>
+    <tableColumn id="9" xr3:uid="{D312A1E1-7C2E-4D8A-944A-4F3689255C0C}" name="Уровень экспертизы"/>
+    <tableColumn id="10" xr3:uid="{7AE2A8AB-0688-4A8B-8012-028FAC792776}" name="Рабочее место"/>
+    <tableColumn id="11" xr3:uid="{E00E5D5B-B0D7-4D3E-8330-D83170ECDFFD}" name="Документ УЛ"/>
+    <tableColumn id="12" xr3:uid="{7856E0FF-220B-4C61-A0A9-7F69D6EEC19E}" name="Адрес по регистрации"/>
+    <tableColumn id="13" xr3:uid="{44810D1B-1CF3-4DCF-83FF-EA7B1EED8C28}" name="Пол"/>
+    <tableColumn id="14" xr3:uid="{AD618D33-9F1F-4128-82F7-EFFB19B34980}" name="ФИО супруга/супруги"/>
+    <tableColumn id="15" xr3:uid="{8E247D4A-8763-4FAF-A7A3-EC126825E3BF}" name="Рабочий день"/>
+    <tableColumn id="16" xr3:uid="{B1BA21C0-74F6-4B20-9CB0-AD84D7F04623}" name="Место работы"/>
+    <tableColumn id="18" xr3:uid="{6AFC2477-2AC6-4181-97C1-55DE239AB899}" name="Город проживания"/>
+    <tableColumn id="19" xr3:uid="{5B31A27F-B1A8-49A9-85BF-1C34811AF3DC}" name="Дети"/>
+    <tableColumn id="20" xr3:uid="{512F8F09-CC0D-4E0A-93C2-9B4E67614C53}" name="Семейный статус"/>
+    <tableColumn id="21" xr3:uid="{AD98EEC2-5FB0-4A32-969B-092FF90D08BC}" name="Загранпаспорт"/>
+    <tableColumn id="22" xr3:uid="{213A8395-60CF-4627-8BFA-8B7932AB04B3}" name="Уровень английского"/>
+    <tableColumn id="23" xr3:uid="{2B2BC760-206D-4B47-91E1-3A23B46C94A0}" name="Дата увольнения" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Таблица1" displayName="Таблица1" ref="A3:E4" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A3:E4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:E4">
+    <sortCondition ref="A3:A4"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ФИО сотрудника"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email сотрудника" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Имя ребёнка" dataDxfId="2"/>
+    <tableColumn id="26" xr3:uid="{2CF1E783-42FA-435B-A9B0-71CCC889D77B}" name="Дата рождения" dataDxfId="0"/>
+    <tableColumn id="24" xr3:uid="{D293F5E8-02A4-47F1-A8B5-1446B2110421}" name="Возраст" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Стандартная">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -587,9 +773,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -622,9 +808,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -657,9 +860,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Стандартная">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -832,8 +1052,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F76F545-ACAE-4135-9050-AC0BC6DE98B0}">
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.5703125" customWidth="1"/>
@@ -860,10 +1080,10 @@
     <col min="24" max="24" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5"/>
       <c r="B1" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -888,7 +1108,7 @@
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="9" t="s">
         <v>1</v>
@@ -918,7 +1138,7 @@
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
     </row>
-    <row r="3" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -929,159 +1149,153 @@
         <v>3</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="V3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="U3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="X3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="Y3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="X3" s="4" t="s">
+      <c r="Z3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Y3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>31</v>
-      </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" t="s">
+        <v>43</v>
+      </c>
+      <c r="O4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S4" t="s">
         <v>38</v>
       </c>
-      <c r="I4" t="s">
-        <v>56</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" t="s">
-        <v>45</v>
-      </c>
-      <c r="O4" t="s">
-        <v>44</v>
-      </c>
-      <c r="P4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>42</v>
-      </c>
-      <c r="R4" t="s">
-        <v>41</v>
-      </c>
-      <c r="S4" t="s">
-        <v>40</v>
-      </c>
       <c r="T4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="U4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="V4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="W4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="X4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Y4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>9</v>
-      </c>
-      <c r="AA4" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="Z4" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1096,10 +1310,77 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CA4589C-B720-4D4E-AE1C-33C6E71A124A}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="41.5703125" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="39.42578125" customWidth="1"/>
+    <col min="4" max="5" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>